<commit_message>
Omit Columns with Policy tag
</commit_message>
<xml_diff>
--- a/dataplex-dq-agent/descriptions/dh1_dq_descriptions_ent_actvn.xlsx
+++ b/dataplex-dq-agent/descriptions/dh1_dq_descriptions_ent_actvn.xlsx
@@ -7292,19 +7292,14 @@
           <t>bq_dly_servreq_actvy_sum_h</t>
         </is>
       </c>
-      <c r="D216" t="inlineStr">
-        <is>
-          <t>This table contains a daily summary of customer service activities, which are transactions that result in modifications to a customer's existing products or services.</t>
-        </is>
-      </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7324,19 +7319,14 @@
           <t>dly_servreq_actvy_sum_ts</t>
         </is>
       </c>
-      <c r="D217" t="inlineStr">
-        <is>
-          <t>This column contains the timestamp when the daily summary record for the service request activity was generated.</t>
-        </is>
-      </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7356,19 +7346,14 @@
           <t>dly_servreq_actvy_sum_key</t>
         </is>
       </c>
-      <c r="D218" t="inlineStr">
-        <is>
-          <t>This column contains the unique system-generated identifier for each daily service request activity summary record.</t>
-        </is>
-      </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7388,19 +7373,14 @@
           <t>dly_servreq_actvy_sum_dt_key</t>
         </is>
       </c>
-      <c r="D219" t="inlineStr">
-        <is>
-          <t>This column contains the key representing the date of the daily summary for the service request activity.</t>
-        </is>
-      </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7420,19 +7400,14 @@
           <t>prod_instnc_key</t>
         </is>
       </c>
-      <c r="D220" t="inlineStr">
-        <is>
-          <t>This column contains the unique system-generated identifier for a specific instance of a product or service.</t>
-        </is>
-      </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7452,19 +7427,14 @@
           <t>cust_key</t>
         </is>
       </c>
-      <c r="D221" t="inlineStr">
-        <is>
-          <t>This column contains the unique system-generated identifier for a customer.</t>
-        </is>
-      </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7484,19 +7454,14 @@
           <t>servreq_action_type_key</t>
         </is>
       </c>
-      <c r="D222" t="inlineStr">
-        <is>
-          <t>This column contains the key that identifies the type of action performed as part of the service request.</t>
-        </is>
-      </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7516,19 +7481,14 @@
           <t>cust_id</t>
         </is>
       </c>
-      <c r="D223" t="inlineStr">
-        <is>
-          <t>This column contains the unique identifier assigned to a customer.</t>
-        </is>
-      </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7548,19 +7508,14 @@
           <t>servreq_header_id</t>
         </is>
       </c>
-      <c r="D224" t="inlineStr">
-        <is>
-          <t>This column contains the unique identifier for the overall service request transaction.</t>
-        </is>
-      </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7580,19 +7535,14 @@
           <t>servreq_header_nm</t>
         </is>
       </c>
-      <c r="D225" t="inlineStr">
-        <is>
-          <t>This column contains the name or title given to the service request.</t>
-        </is>
-      </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7612,19 +7562,14 @@
           <t>servreq_transaction_ts</t>
         </is>
       </c>
-      <c r="D226" t="inlineStr">
-        <is>
-          <t>This column contains the date and time when the service request transaction was executed.</t>
-        </is>
-      </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7644,19 +7589,14 @@
           <t>servreq_event_type_cd</t>
         </is>
       </c>
-      <c r="D227" t="inlineStr">
-        <is>
-          <t>This column contains a code that represents the specific type of event that occurred within the service request.</t>
-        </is>
-      </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7676,19 +7616,14 @@
           <t>servreq_event_type_nm</t>
         </is>
       </c>
-      <c r="D228" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the event that occurred within the service request.</t>
-        </is>
-      </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7708,19 +7643,14 @@
           <t>servreq_header_status_cd</t>
         </is>
       </c>
-      <c r="D229" t="inlineStr">
-        <is>
-          <t>This column contains a code indicating the current status of the overall service request.</t>
-        </is>
-      </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7740,19 +7670,14 @@
           <t>servreq_actor_role_nm</t>
         </is>
       </c>
-      <c r="D230" t="inlineStr">
-        <is>
-          <t>This column contains the role of the person or system that performed the action within the service request.</t>
-        </is>
-      </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7772,19 +7697,14 @@
           <t>prod_instnc_id</t>
         </is>
       </c>
-      <c r="D231" t="inlineStr">
-        <is>
-          <t>This column contains the unique identifier for a specific instance of a product or service subscribed to by a customer.</t>
-        </is>
-      </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7804,19 +7724,14 @@
           <t>prod_instnc_type_cd</t>
         </is>
       </c>
-      <c r="D232" t="inlineStr">
-        <is>
-          <t>This column contains a code that categorizes the type of product instance, such as a mobile phone line or internet service.</t>
-        </is>
-      </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7836,19 +7751,14 @@
           <t>prod_instnc_activation_ts</t>
         </is>
       </c>
-      <c r="D233" t="inlineStr">
-        <is>
-          <t>This column contains the date and time when the specific product or service instance was first activated.</t>
-        </is>
-      </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7868,19 +7778,14 @@
           <t>prim_srvc_resrc_str</t>
         </is>
       </c>
-      <c r="D234" t="inlineStr">
-        <is>
-          <t>This column contains the primary resource associated with the service, such as a phone number or account identifier.</t>
-        </is>
-      </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7900,19 +7805,14 @@
           <t>brand_cd</t>
         </is>
       </c>
-      <c r="D235" t="inlineStr">
-        <is>
-          <t>This column contains a code representing the TELUS brand under which the product or service is offered.</t>
-        </is>
-      </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7932,19 +7832,14 @@
           <t>brand_txt</t>
         </is>
       </c>
-      <c r="D236" t="inlineStr">
-        <is>
-          <t>This column contains the name of the TELUS brand associated with the product or service.</t>
-        </is>
-      </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7964,19 +7859,14 @@
           <t>bacct_num</t>
         </is>
       </c>
-      <c r="D237" t="inlineStr">
-        <is>
-          <t>This column contains the unique number assigned to the customer's billing account.</t>
-        </is>
-      </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -7996,19 +7886,14 @@
           <t>billing_acct_status_cd</t>
         </is>
       </c>
-      <c r="D238" t="inlineStr">
-        <is>
-          <t>This column contains a code representing the current status of the customer's billing account.</t>
-        </is>
-      </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8028,19 +7913,14 @@
           <t>billing_acct_status_txt</t>
         </is>
       </c>
-      <c r="D239" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive text for the current status of the customer's billing account.</t>
-        </is>
-      </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8060,19 +7940,14 @@
           <t>billing_account_type_cd</t>
         </is>
       </c>
-      <c r="D240" t="inlineStr">
-        <is>
-          <t>This column contains a code that categorizes the type of billing account, such as personal or business.</t>
-        </is>
-      </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8092,19 +7967,14 @@
           <t>billing_account_type_txt</t>
         </is>
       </c>
-      <c r="D241" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the billing account type.</t>
-        </is>
-      </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8124,19 +7994,14 @@
           <t>billing_account_subtype_cd</t>
         </is>
       </c>
-      <c r="D242" t="inlineStr">
-        <is>
-          <t>This column contains a code that provides a more detailed classification of the billing account type.</t>
-        </is>
-      </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8156,19 +8021,14 @@
           <t>billing_account_subtype_txt</t>
         </is>
       </c>
-      <c r="D243" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the billing account subtype.</t>
-        </is>
-      </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8188,19 +8048,14 @@
           <t>billing_cycle_cd</t>
         </is>
       </c>
-      <c r="D244" t="inlineStr">
-        <is>
-          <t>This column contains a code representing the customer's billing frequency and schedule.</t>
-        </is>
-      </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8220,19 +8075,14 @@
           <t>billing_cycle_txt</t>
         </is>
       </c>
-      <c r="D245" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the customer's billing cycle.</t>
-        </is>
-      </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8252,19 +8102,14 @@
           <t>segment_type_cd</t>
         </is>
       </c>
-      <c r="D246" t="inlineStr">
-        <is>
-          <t>This column contains a code used to classify the customer into a specific market segment.</t>
-        </is>
-      </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8284,19 +8129,14 @@
           <t>segment_type_txt</t>
         </is>
       </c>
-      <c r="D247" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the customer's market segment.</t>
-        </is>
-      </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8316,19 +8156,14 @@
           <t>ilec_segment_type_cd</t>
         </is>
       </c>
-      <c r="D248" t="inlineStr">
-        <is>
-          <t>This column contains a code for the customer segment within the Incumbent Local Exchange Carrier business context.</t>
-        </is>
-      </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8348,19 +8183,14 @@
           <t>ilec_segment_type_txt</t>
         </is>
       </c>
-      <c r="D249" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the customer segment within the Incumbent Local Exchange Carrier business context.</t>
-        </is>
-      </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8380,19 +8210,14 @@
           <t>govt_segment_type_cd</t>
         </is>
       </c>
-      <c r="D250" t="inlineStr">
-        <is>
-          <t>This column contains a code used to classify a customer within a government market segment.</t>
-        </is>
-      </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8412,19 +8237,14 @@
           <t>govt_segment_type_txt</t>
         </is>
       </c>
-      <c r="D251" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the government market segment.</t>
-        </is>
-      </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8444,19 +8264,14 @@
           <t>segment_group_cd</t>
         </is>
       </c>
-      <c r="D252" t="inlineStr">
-        <is>
-          <t>This column contains a code for a broader grouping of customer market segments.</t>
-        </is>
-      </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8476,19 +8291,14 @@
           <t>segment_group_txt</t>
         </is>
       </c>
-      <c r="D253" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the broader customer market segment group.</t>
-        </is>
-      </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8508,19 +8318,14 @@
           <t>segment_minor_group_cd</t>
         </is>
       </c>
-      <c r="D254" t="inlineStr">
-        <is>
-          <t>This column contains a code for a more granular grouping within a customer segment group.</t>
-        </is>
-      </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8540,19 +8345,14 @@
           <t>segment_minor_group_txt</t>
         </is>
       </c>
-      <c r="D255" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the minor customer segment group.</t>
-        </is>
-      </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8572,19 +8372,14 @@
           <t>revenue_band_type_cd</t>
         </is>
       </c>
-      <c r="D256" t="inlineStr">
-        <is>
-          <t>This column contains a code that classifies the customer based on their level of spending.</t>
-        </is>
-      </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8604,19 +8399,14 @@
           <t>combo_group_id</t>
         </is>
       </c>
-      <c r="D257" t="inlineStr">
-        <is>
-          <t>This column contains the identifier for a group of bundled products or services.</t>
-        </is>
-      </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8636,19 +8426,14 @@
           <t>combo_group_txt</t>
         </is>
       </c>
-      <c r="D258" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the group of bundled products or services.</t>
-        </is>
-      </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8668,19 +8453,14 @@
           <t>prod_instnc_cnt</t>
         </is>
       </c>
-      <c r="D259" t="inlineStr">
-        <is>
-          <t>This column contains the total count of product instances associated with the customer's account.</t>
-        </is>
-      </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8700,19 +8480,14 @@
           <t>combo_prod_instnc_cnt</t>
         </is>
       </c>
-      <c r="D260" t="inlineStr">
-        <is>
-          <t>This column contains the count of product instances that are part of a bundled offer.</t>
-        </is>
-      </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8732,19 +8507,14 @@
           <t>new_handset_serial_num</t>
         </is>
       </c>
-      <c r="D261" t="inlineStr">
-        <is>
-          <t>This column contains the serial number of the new device involved in the service request.</t>
-        </is>
-      </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8764,19 +8534,14 @@
           <t>old_handset_serial_num</t>
         </is>
       </c>
-      <c r="D262" t="inlineStr">
-        <is>
-          <t>This column contains the serial number of the previous device that was replaced or modified.</t>
-        </is>
-      </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8796,19 +8561,14 @@
           <t>new_handset_product_cd</t>
         </is>
       </c>
-      <c r="D263" t="inlineStr">
-        <is>
-          <t>This column contains the product code that identifies the new handset or device.</t>
-        </is>
-      </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8828,19 +8588,14 @@
           <t>old_handset_product_cd</t>
         </is>
       </c>
-      <c r="D264" t="inlineStr">
-        <is>
-          <t>This column contains the product code that identifies the previous handset or device.</t>
-        </is>
-      </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8860,19 +8615,14 @@
           <t>handset_mtm_price_amt</t>
         </is>
       </c>
-      <c r="D265" t="inlineStr">
-        <is>
-          <t>This column contains the month-to-month price of the handset without a contract term.</t>
-        </is>
-      </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8892,19 +8642,14 @@
           <t>sim_serial_num</t>
         </is>
       </c>
-      <c r="D266" t="inlineStr">
-        <is>
-          <t>This column contains the unique serial number of the Subscriber Identity Module card.</t>
-        </is>
-      </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8924,19 +8669,14 @@
           <t>sim_product_cd</t>
         </is>
       </c>
-      <c r="D267" t="inlineStr">
-        <is>
-          <t>This column contains the product code that identifies the Subscriber Identity Module card.</t>
-        </is>
-      </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8956,19 +8696,14 @@
           <t>outlet_id</t>
         </is>
       </c>
-      <c r="D268" t="inlineStr">
-        <is>
-          <t>This column contains the unique identifier for the sales outlet where the transaction occurred.</t>
-        </is>
-      </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -8988,19 +8723,14 @@
           <t>outlet_cd</t>
         </is>
       </c>
-      <c r="D269" t="inlineStr">
-        <is>
-          <t>This column contains the code that represents the specific sales outlet.</t>
-        </is>
-      </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9020,19 +8750,14 @@
           <t>outlet_txt</t>
         </is>
       </c>
-      <c r="D270" t="inlineStr">
-        <is>
-          <t>This column contains the name of the sales outlet where the transaction occurred.</t>
-        </is>
-      </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9052,19 +8777,14 @@
           <t>outlet_type_cd</t>
         </is>
       </c>
-      <c r="D271" t="inlineStr">
-        <is>
-          <t>This column contains a code that categorizes the type of sales outlet, such as a corporate store or dealer.</t>
-        </is>
-      </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9084,19 +8804,14 @@
           <t>outlet_sales_type_cd</t>
         </is>
       </c>
-      <c r="D272" t="inlineStr">
-        <is>
-          <t>This column contains a code that categorizes the type of sale made at the outlet.</t>
-        </is>
-      </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9116,19 +8831,14 @@
           <t>outlet_province_cd</t>
         </is>
       </c>
-      <c r="D273" t="inlineStr">
-        <is>
-          <t>This column contains the code for the province where the sales outlet is located.</t>
-        </is>
-      </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9148,19 +8858,14 @@
           <t>outlet_city_nm</t>
         </is>
       </c>
-      <c r="D274" t="inlineStr">
-        <is>
-          <t>This column contains the name of the city where the sales outlet is located.</t>
-        </is>
-      </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9180,19 +8885,14 @@
           <t>outlet_country_cd</t>
         </is>
       </c>
-      <c r="D275" t="inlineStr">
-        <is>
-          <t>This column contains the code for the country where the sales outlet is located.</t>
-        </is>
-      </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9212,19 +8912,14 @@
           <t>outlet_postal_cd</t>
         </is>
       </c>
-      <c r="D276" t="inlineStr">
-        <is>
-          <t>This column contains the postal code of the sales outlet's location.</t>
-        </is>
-      </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9244,19 +8939,14 @@
           <t>outlet_street_num</t>
         </is>
       </c>
-      <c r="D277" t="inlineStr">
-        <is>
-          <t>This column contains the street number of the sales outlet's address.</t>
-        </is>
-      </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9276,19 +8966,14 @@
           <t>outlet_street_nm</t>
         </is>
       </c>
-      <c r="D278" t="inlineStr">
-        <is>
-          <t>This column contains the street name of the sales outlet's address.</t>
-        </is>
-      </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9308,19 +8993,14 @@
           <t>outlet_street_prefix_cd</t>
         </is>
       </c>
-      <c r="D279" t="inlineStr">
-        <is>
-          <t>This column contains the directional prefix for the street name in the sales outlet's address.</t>
-        </is>
-      </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9340,19 +9020,14 @@
           <t>outlet_street_type_cd</t>
         </is>
       </c>
-      <c r="D280" t="inlineStr">
-        <is>
-          <t>This column contains the type of street, such as 'Street' or 'Avenue', in the sales outlet's address.</t>
-        </is>
-      </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9372,19 +9047,14 @@
           <t>chnl_org_id</t>
         </is>
       </c>
-      <c r="D281" t="inlineStr">
-        <is>
-          <t>This column contains the unique identifier for the sales channel organization.</t>
-        </is>
-      </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9404,19 +9074,14 @@
           <t>chnl_org_cd</t>
         </is>
       </c>
-      <c r="D282" t="inlineStr">
-        <is>
-          <t>This column contains the code that represents the sales channel organization.</t>
-        </is>
-      </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9436,19 +9101,14 @@
           <t>chnl_org_txt</t>
         </is>
       </c>
-      <c r="D283" t="inlineStr">
-        <is>
-          <t>This column contains the name of the sales channel organization.</t>
-        </is>
-      </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9468,19 +9128,14 @@
           <t>chnl_org_type_cd</t>
         </is>
       </c>
-      <c r="D284" t="inlineStr">
-        <is>
-          <t>This column contains a code that categorizes the type of sales channel organization.</t>
-        </is>
-      </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9500,19 +9155,14 @@
           <t>chnl_org_type_txt</t>
         </is>
       </c>
-      <c r="D285" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the sales channel organization type.</t>
-        </is>
-      </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9532,19 +9182,14 @@
           <t>sales_rep_id</t>
         </is>
       </c>
-      <c r="D286" t="inlineStr">
-        <is>
-          <t>This column contains the unique identifier for the sales representative who handled the transaction.</t>
-        </is>
-      </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9564,19 +9209,14 @@
           <t>sales_rep_cd</t>
         </is>
       </c>
-      <c r="D287" t="inlineStr">
-        <is>
-          <t>This column contains the code assigned to the sales representative.</t>
-        </is>
-      </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9596,19 +9236,14 @@
           <t>sales_rep_first_nm</t>
         </is>
       </c>
-      <c r="D288" t="inlineStr">
-        <is>
-          <t>This column contains the first name of the sales representative.</t>
-        </is>
-      </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9628,19 +9263,14 @@
           <t>sales_rep_last_nm</t>
         </is>
       </c>
-      <c r="D289" t="inlineStr">
-        <is>
-          <t>This column contains the last name of the sales representative.</t>
-        </is>
-      </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9660,19 +9290,14 @@
           <t>kb_sales_rep_cd</t>
         </is>
       </c>
-      <c r="D290" t="inlineStr">
-        <is>
-          <t>This column contains the sales representative code from the Koodo brand system.</t>
-        </is>
-      </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9692,19 +9317,14 @@
           <t>kb_dealer_cd</t>
         </is>
       </c>
-      <c r="D291" t="inlineStr">
-        <is>
-          <t>This column contains the dealer code from the Koodo brand system.</t>
-        </is>
-      </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9724,19 +9344,14 @@
           <t>offer_discount_amt</t>
         </is>
       </c>
-      <c r="D292" t="inlineStr">
-        <is>
-          <t>This column contains the total discount amount applied as part of a specific offer.</t>
-        </is>
-      </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9756,19 +9371,14 @@
           <t>term_discount_amt</t>
         </is>
       </c>
-      <c r="D293" t="inlineStr">
-        <is>
-          <t>This column contains the discount amount applied to the customer's account related to their contract term.</t>
-        </is>
-      </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9788,19 +9398,14 @@
           <t>other_discount_amt</t>
         </is>
       </c>
-      <c r="D294" t="inlineStr">
-        <is>
-          <t>This column contains the value of any miscellaneous discounts applied to the transaction.</t>
-        </is>
-      </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9820,19 +9425,14 @@
           <t>dvc_bal_chrg_amt</t>
         </is>
       </c>
-      <c r="D295" t="inlineStr">
-        <is>
-          <t>This column contains the amount charged to the customer for their remaining device balance.</t>
-        </is>
-      </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9852,19 +9452,14 @@
           <t>dvc_bal_waive_amt</t>
         </is>
       </c>
-      <c r="D296" t="inlineStr">
-        <is>
-          <t>This column contains the amount of the customer's remaining device balance that was waived.</t>
-        </is>
-      </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9884,19 +9479,14 @@
           <t>promotion_type_cd</t>
         </is>
       </c>
-      <c r="D297" t="inlineStr">
-        <is>
-          <t>This column contains a code that categorizes the type of promotion applied to the transaction.</t>
-        </is>
-      </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9916,19 +9506,14 @@
           <t>offer_cd</t>
         </is>
       </c>
-      <c r="D298" t="inlineStr">
-        <is>
-          <t>This column contains the code that uniquely identifies the offer applied to the service.</t>
-        </is>
-      </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9948,19 +9533,14 @@
           <t>offer_txt</t>
         </is>
       </c>
-      <c r="D299" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the offer applied to the service.</t>
-        </is>
-      </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9980,19 +9560,14 @@
           <t>mktg_pgm_cd</t>
         </is>
       </c>
-      <c r="D300" t="inlineStr">
-        <is>
-          <t>This column contains a code identifying the marketing program associated with the transaction.</t>
-        </is>
-      </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10012,19 +9587,14 @@
           <t>activation_offer_id</t>
         </is>
       </c>
-      <c r="D301" t="inlineStr">
-        <is>
-          <t>This column contains the unique identifier for the offer applied at the time of service activation.</t>
-        </is>
-      </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10044,19 +9614,14 @@
           <t>renewal_offer_id</t>
         </is>
       </c>
-      <c r="D302" t="inlineStr">
-        <is>
-          <t>This column contains the unique identifier for the offer applied at the time of service renewal.</t>
-        </is>
-      </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10076,19 +9641,14 @@
           <t>offer_group_txt</t>
         </is>
       </c>
-      <c r="D303" t="inlineStr">
-        <is>
-          <t>This column contains the name of the group to which the specific offer belongs.</t>
-        </is>
-      </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10108,19 +9668,14 @@
           <t>new_contract_start_dt</t>
         </is>
       </c>
-      <c r="D304" t="inlineStr">
-        <is>
-          <t>This column contains the start date of the new service agreement.</t>
-        </is>
-      </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10140,19 +9695,14 @@
           <t>old_contract_start_dt</t>
         </is>
       </c>
-      <c r="D305" t="inlineStr">
-        <is>
-          <t>This column contains the start date of the previous service agreement.</t>
-        </is>
-      </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10172,19 +9722,14 @@
           <t>new_contract_end_dt</t>
         </is>
       </c>
-      <c r="D306" t="inlineStr">
-        <is>
-          <t>This column contains the end date of the new service agreement.</t>
-        </is>
-      </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10204,19 +9749,14 @@
           <t>old_contract_end_dt</t>
         </is>
       </c>
-      <c r="D307" t="inlineStr">
-        <is>
-          <t>This column contains the end date of the previous service agreement.</t>
-        </is>
-      </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10236,19 +9776,14 @@
           <t>new_contract_months_cnt</t>
         </is>
       </c>
-      <c r="D308" t="inlineStr">
-        <is>
-          <t>This column contains the duration of the new service agreement in months.</t>
-        </is>
-      </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10268,19 +9803,14 @@
           <t>old_contract_months_cnt</t>
         </is>
       </c>
-      <c r="D309" t="inlineStr">
-        <is>
-          <t>This column contains the duration of the previous service agreement in months.</t>
-        </is>
-      </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10300,19 +9830,14 @@
           <t>new_pp_catlg_cd</t>
         </is>
       </c>
-      <c r="D310" t="inlineStr">
-        <is>
-          <t>This column contains the catalog code for the customer's new price plan.</t>
-        </is>
-      </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10332,19 +9857,14 @@
           <t>new_price_plan_txt</t>
         </is>
       </c>
-      <c r="D311" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the customer's new price plan.</t>
-        </is>
-      </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10364,19 +9884,14 @@
           <t>old_pp_catlg_cd</t>
         </is>
       </c>
-      <c r="D312" t="inlineStr">
-        <is>
-          <t>This column contains the catalog code for the customer's previous price plan.</t>
-        </is>
-      </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10396,19 +9911,14 @@
           <t>old_price_plan_txt</t>
         </is>
       </c>
-      <c r="D313" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the customer's previous price plan.</t>
-        </is>
-      </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10428,19 +9938,14 @@
           <t>new_prepaid_ind</t>
         </is>
       </c>
-      <c r="D314" t="inlineStr">
-        <is>
-          <t>This column contains a yes/no indicator identifying if the new plan is a prepaid plan.</t>
-        </is>
-      </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10460,19 +9965,14 @@
           <t>old_prepaid_ind</t>
         </is>
       </c>
-      <c r="D315" t="inlineStr">
-        <is>
-          <t>This column contains a yes/no indicator identifying if the previous plan was a prepaid plan.</t>
-        </is>
-      </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10492,19 +9992,14 @@
           <t>new_revenue_ind</t>
         </is>
       </c>
-      <c r="D316" t="inlineStr">
-        <is>
-          <t>This column contains a yes/no indicator identifying if the new plan is considered revenue-generating.</t>
-        </is>
-      </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10524,19 +10019,14 @@
           <t>old_revenue_ind</t>
         </is>
       </c>
-      <c r="D317" t="inlineStr">
-        <is>
-          <t>This column contains a yes/no indicator identifying if the previous plan was considered revenue-generating.</t>
-        </is>
-      </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10556,19 +10046,14 @@
           <t>new_price_plan_rate_amt</t>
         </is>
       </c>
-      <c r="D318" t="inlineStr">
-        <is>
-          <t>This column contains the base rate amount for the new price plan.</t>
-        </is>
-      </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10588,19 +10073,14 @@
           <t>old_price_plan_rate_amt</t>
         </is>
       </c>
-      <c r="D319" t="inlineStr">
-        <is>
-          <t>This column contains the base rate amount for the previous price plan.</t>
-        </is>
-      </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10620,19 +10100,14 @@
           <t>new_feature_charge_amt</t>
         </is>
       </c>
-      <c r="D320" t="inlineStr">
-        <is>
-          <t>This column contains the total amount charged for add-on features on the new plan.</t>
-        </is>
-      </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10652,19 +10127,14 @@
           <t>old_feature_charge_amt</t>
         </is>
       </c>
-      <c r="D321" t="inlineStr">
-        <is>
-          <t>This column contains the total amount charged for add-on features on the previous plan.</t>
-        </is>
-      </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10684,19 +10154,14 @@
           <t>new_mrc_amt</t>
         </is>
       </c>
-      <c r="D322" t="inlineStr">
-        <is>
-          <t>This column contains the new total monthly recurring charge for the customer's services.</t>
-        </is>
-      </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10716,19 +10181,14 @@
           <t>old_mrc_amt</t>
         </is>
       </c>
-      <c r="D323" t="inlineStr">
-        <is>
-          <t>This column contains the previous total monthly recurring charge for the customer's services.</t>
-        </is>
-      </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10748,19 +10208,14 @@
           <t>mrc_calculation_dt</t>
         </is>
       </c>
-      <c r="D324" t="inlineStr">
-        <is>
-          <t>This column contains the date on which the monthly recurring charge was calculated.</t>
-        </is>
-      </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10780,19 +10235,14 @@
           <t>hardware_discount_amt</t>
         </is>
       </c>
-      <c r="D325" t="inlineStr">
-        <is>
-          <t>This column contains the discount amount applied to the hardware or device.</t>
-        </is>
-      </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10812,19 +10262,14 @@
           <t>mth_from_contract_start_cnt</t>
         </is>
       </c>
-      <c r="D326" t="inlineStr">
-        <is>
-          <t>This column contains the number of months that have passed since the contract start date.</t>
-        </is>
-      </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10844,19 +10289,14 @@
           <t>mth_to_expiry_cnt</t>
         </is>
       </c>
-      <c r="D327" t="inlineStr">
-        <is>
-          <t>This column contains the number of months remaining until the contract expires.</t>
-        </is>
-      </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10876,19 +10316,14 @@
           <t>new_prod_catlg_item_intrn_nm</t>
         </is>
       </c>
-      <c r="D328" t="inlineStr">
-        <is>
-          <t>This column contains the internal name for the new product from the product catalog.</t>
-        </is>
-      </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10908,19 +10343,14 @@
           <t>old_prod_catlg_item_intrn_nm</t>
         </is>
       </c>
-      <c r="D329" t="inlineStr">
-        <is>
-          <t>This column contains the internal name for the previous product from the product catalog.</t>
-        </is>
-      </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10940,19 +10370,14 @@
           <t>new_prod_equip_mfr_nm</t>
         </is>
       </c>
-      <c r="D330" t="inlineStr">
-        <is>
-          <t>This column contains the name of the manufacturer of the new equipment or device.</t>
-        </is>
-      </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -10972,19 +10397,14 @@
           <t>old_prod_equip_mfr_nm</t>
         </is>
       </c>
-      <c r="D331" t="inlineStr">
-        <is>
-          <t>This column contains the name of the manufacturer of the previous equipment or device.</t>
-        </is>
-      </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11004,19 +10424,14 @@
           <t>new_prod_equip_tech_type_cd</t>
         </is>
       </c>
-      <c r="D332" t="inlineStr">
-        <is>
-          <t>This column contains a code for the technology type of the new equipment, such as 5G or LTE.</t>
-        </is>
-      </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11036,19 +10451,14 @@
           <t>new_prod_equip_tech_type_txt</t>
         </is>
       </c>
-      <c r="D333" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the technology type for the new equipment.</t>
-        </is>
-      </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11068,19 +10478,14 @@
           <t>old_prod_equip_tech_type_cd</t>
         </is>
       </c>
-      <c r="D334" t="inlineStr">
-        <is>
-          <t>This column contains a code for the technology type of the previous equipment, such as 5G or LTE.</t>
-        </is>
-      </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11100,19 +10505,14 @@
           <t>old_prod_equip_tech_type_txt</t>
         </is>
       </c>
-      <c r="D335" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the technology type for the previous equipment.</t>
-        </is>
-      </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11132,19 +10532,14 @@
           <t>new_handset_platform_nm</t>
         </is>
       </c>
-      <c r="D336" t="inlineStr">
-        <is>
-          <t>This column contains the name of the operating system platform of the new handset.</t>
-        </is>
-      </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11164,19 +10559,14 @@
           <t>old_handset_platform_nm</t>
         </is>
       </c>
-      <c r="D337" t="inlineStr">
-        <is>
-          <t>This column contains the name of the operating system platform of the previous handset.</t>
-        </is>
-      </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11196,19 +10586,14 @@
           <t>new_handset_type_nm</t>
         </is>
       </c>
-      <c r="D338" t="inlineStr">
-        <is>
-          <t>This column contains the type or category of the new handset, such as smartphone or feature phone.</t>
-        </is>
-      </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11228,19 +10613,14 @@
           <t>old_handset_type_nm</t>
         </is>
       </c>
-      <c r="D339" t="inlineStr">
-        <is>
-          <t>This column contains the type or category of the previous handset, such as smartphone or feature phone.</t>
-        </is>
-      </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11260,19 +10640,14 @@
           <t>rate_area_centre_cd</t>
         </is>
       </c>
-      <c r="D340" t="inlineStr">
-        <is>
-          <t>This column contains a code identifying the geographic rate center for billing purposes.</t>
-        </is>
-      </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11292,19 +10667,14 @@
           <t>rate_area_centre_txt</t>
         </is>
       </c>
-      <c r="D341" t="inlineStr">
-        <is>
-          <t>This column contains the name of the geographic rate center.</t>
-        </is>
-      </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11324,19 +10694,14 @@
           <t>rate_area_centre_prov_cd</t>
         </is>
       </c>
-      <c r="D342" t="inlineStr">
-        <is>
-          <t>This column contains the province code for the geographic rate center.</t>
-        </is>
-      </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11356,19 +10721,14 @@
           <t>rate_area_market_cd</t>
         </is>
       </c>
-      <c r="D343" t="inlineStr">
-        <is>
-          <t>This column contains a code for the market associated with the geographic rate area.</t>
-        </is>
-      </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11388,19 +10748,14 @@
           <t>rate_area_sub_market_cd</t>
         </is>
       </c>
-      <c r="D344" t="inlineStr">
-        <is>
-          <t>This column contains a code for the sub-market associated with the geographic rate area.</t>
-        </is>
-      </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11420,19 +10775,14 @@
           <t>rate_area_region_cd</t>
         </is>
       </c>
-      <c r="D345" t="inlineStr">
-        <is>
-          <t>This column contains a code for the region associated with the geographic rate area.</t>
-        </is>
-      </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11452,19 +10802,14 @@
           <t>payment_responsible_ind</t>
         </is>
       </c>
-      <c r="D346" t="inlineStr">
-        <is>
-          <t>This column contains a yes/no indicator identifying if the customer associated with this service is responsible for payment.</t>
-        </is>
-      </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11484,19 +10829,14 @@
           <t>sales_region_seg_type_cd</t>
         </is>
       </c>
-      <c r="D347" t="inlineStr">
-        <is>
-          <t>This column contains a code for the customer segment within a specific sales region.</t>
-        </is>
-      </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11516,19 +10856,14 @@
           <t>sales_region_seg_type_txt</t>
         </is>
       </c>
-      <c r="D348" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the customer segment within a specific sales region.</t>
-        </is>
-      </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F348" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11548,19 +10883,14 @@
           <t>paper_invoice_ind</t>
         </is>
       </c>
-      <c r="D349" t="inlineStr">
-        <is>
-          <t>This column contains a yes/no indicator identifying if the customer receives a paper invoice.</t>
-        </is>
-      </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11580,19 +10910,14 @@
           <t>indvdl_first_nm</t>
         </is>
       </c>
-      <c r="D350" t="inlineStr">
-        <is>
-          <t>This column contains the first name of the individual customer.</t>
-        </is>
-      </c>
       <c r="E350" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F350" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11612,19 +10937,14 @@
           <t>indvdl_last_nm</t>
         </is>
       </c>
-      <c r="D351" t="inlineStr">
-        <is>
-          <t>This column contains the last name of the individual customer.</t>
-        </is>
-      </c>
       <c r="E351" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F351" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11644,19 +10964,14 @@
           <t>acct_activation_ts</t>
         </is>
       </c>
-      <c r="D352" t="inlineStr">
-        <is>
-          <t>This column contains the date the customer's account was originally activated.</t>
-        </is>
-      </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F352" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11676,19 +10991,14 @@
           <t>prod_instnc_postal_cd</t>
         </is>
       </c>
-      <c r="D353" t="inlineStr">
-        <is>
-          <t>This column contains the postal code associated with the service location of the product instance.</t>
-        </is>
-      </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11708,19 +11018,14 @@
           <t>prod_instnc_prov_state_cd</t>
         </is>
       </c>
-      <c r="D354" t="inlineStr">
-        <is>
-          <t>This column contains the province or state code for the service location of the product instance.</t>
-        </is>
-      </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11740,19 +11045,14 @@
           <t>processing_eligibility_num</t>
         </is>
       </c>
-      <c r="D355" t="inlineStr">
-        <is>
-          <t>This column contains a number used to determine eligibility for transaction processing.</t>
-        </is>
-      </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11772,19 +11072,14 @@
           <t>aom_id</t>
         </is>
       </c>
-      <c r="D356" t="inlineStr">
-        <is>
-          <t>This column contains the unique identifier for a specific marketing offer.</t>
-        </is>
-      </c>
       <c r="E356" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11804,19 +11099,14 @@
           <t>aom_cd</t>
         </is>
       </c>
-      <c r="D357" t="inlineStr">
-        <is>
-          <t>This column contains the code that represents a specific marketing offer.</t>
-        </is>
-      </c>
       <c r="E357" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11836,19 +11126,14 @@
           <t>aom_txt</t>
         </is>
       </c>
-      <c r="D358" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of a specific marketing offer.</t>
-        </is>
-      </c>
       <c r="E358" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11868,19 +11153,14 @@
           <t>mktg_offer_tier_cd</t>
         </is>
       </c>
-      <c r="D359" t="inlineStr">
-        <is>
-          <t>This column contains a code representing the tier or level of the marketing offer.</t>
-        </is>
-      </c>
       <c r="E359" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11900,19 +11180,14 @@
           <t>mktg_offer_tier_txt</t>
         </is>
       </c>
-      <c r="D360" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the marketing offer tier.</t>
-        </is>
-      </c>
       <c r="E360" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11932,19 +11207,14 @@
           <t>mktg_offer_bib_amt</t>
         </is>
       </c>
-      <c r="D361" t="inlineStr">
-        <is>
-          <t>This column contains the amount associated with the Bring-It-Back program for this marketing offer.</t>
-        </is>
-      </c>
       <c r="E361" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11964,19 +11234,14 @@
           <t>mktg_offer_finance_amt</t>
         </is>
       </c>
-      <c r="D362" t="inlineStr">
-        <is>
-          <t>This column contains the amount being financed as part of the marketing offer.</t>
-        </is>
-      </c>
       <c r="E362" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -11996,19 +11261,14 @@
           <t>mktg_offer_subsidy_amt</t>
         </is>
       </c>
-      <c r="D363" t="inlineStr">
-        <is>
-          <t>This column contains the subsidy amount provided as part of the marketing offer.</t>
-        </is>
-      </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12028,19 +11288,14 @@
           <t>device_upfront_payment_amt</t>
         </is>
       </c>
-      <c r="D364" t="inlineStr">
-        <is>
-          <t>This column contains the amount paid by the customer for the device at the time of the transaction.</t>
-        </is>
-      </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12060,19 +11315,14 @@
           <t>mktg_offer_other_type1</t>
         </is>
       </c>
-      <c r="D365" t="inlineStr">
-        <is>
-          <t>This column contains the type of the first additional component of the marketing offer.</t>
-        </is>
-      </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12092,19 +11342,14 @@
           <t>mktg_offer_other_amt1</t>
         </is>
       </c>
-      <c r="D366" t="inlineStr">
-        <is>
-          <t>This column contains the monetary value of the first additional component of the marketing offer.</t>
-        </is>
-      </c>
       <c r="E366" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12124,19 +11369,14 @@
           <t>mktg_offer_other_type2</t>
         </is>
       </c>
-      <c r="D367" t="inlineStr">
-        <is>
-          <t>This column contains the type of the second additional component of the marketing offer.</t>
-        </is>
-      </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12156,19 +11396,14 @@
           <t>mktg_offer_other_amt2</t>
         </is>
       </c>
-      <c r="D368" t="inlineStr">
-        <is>
-          <t>This column contains the monetary value of the second additional component of the marketing offer.</t>
-        </is>
-      </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12188,19 +11423,14 @@
           <t>mktg_offer_other_type3</t>
         </is>
       </c>
-      <c r="D369" t="inlineStr">
-        <is>
-          <t>This column contains the type of the third additional component of the marketing offer.</t>
-        </is>
-      </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12220,19 +11450,14 @@
           <t>mktg_offer_other_amt3</t>
         </is>
       </c>
-      <c r="D370" t="inlineStr">
-        <is>
-          <t>This column contains the monetary value of the third additional component of the marketing offer.</t>
-        </is>
-      </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12252,19 +11477,14 @@
           <t>mktg_promotion_intrnl_id1</t>
         </is>
       </c>
-      <c r="D371" t="inlineStr">
-        <is>
-          <t>This column contains the internal identifier for the first associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12284,19 +11504,14 @@
           <t>mktg_promotion_cd1</t>
         </is>
       </c>
-      <c r="D372" t="inlineStr">
-        <is>
-          <t>This column contains the code for the first associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12316,19 +11531,14 @@
           <t>mktg_promotion_txt1</t>
         </is>
       </c>
-      <c r="D373" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the first associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E373" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12348,19 +11558,14 @@
           <t>mktg_promotion_amt1</t>
         </is>
       </c>
-      <c r="D374" t="inlineStr">
-        <is>
-          <t>This column contains the monetary value of the first associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12380,19 +11585,14 @@
           <t>mktg_promotion_intrnl_id2</t>
         </is>
       </c>
-      <c r="D375" t="inlineStr">
-        <is>
-          <t>This column contains the internal identifier for the second associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12412,19 +11612,14 @@
           <t>mktg_promotion_cd2</t>
         </is>
       </c>
-      <c r="D376" t="inlineStr">
-        <is>
-          <t>This column contains the code for the second associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12444,19 +11639,14 @@
           <t>mktg_promotion_txt2</t>
         </is>
       </c>
-      <c r="D377" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the second associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12476,19 +11666,14 @@
           <t>mktg_promotion_amt2</t>
         </is>
       </c>
-      <c r="D378" t="inlineStr">
-        <is>
-          <t>This column contains the monetary value of the second associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12508,19 +11693,14 @@
           <t>mktg_promotion_intrnl_id3</t>
         </is>
       </c>
-      <c r="D379" t="inlineStr">
-        <is>
-          <t>This column contains the internal identifier for the third associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E379" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12540,19 +11720,14 @@
           <t>mktg_promotion_cd3</t>
         </is>
       </c>
-      <c r="D380" t="inlineStr">
-        <is>
-          <t>This column contains the code for the third associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E380" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12572,19 +11747,14 @@
           <t>mktg_promotion_txt3</t>
         </is>
       </c>
-      <c r="D381" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the third associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E381" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12604,19 +11774,14 @@
           <t>mktg_promotion_amt3</t>
         </is>
       </c>
-      <c r="D382" t="inlineStr">
-        <is>
-          <t>This column contains the monetary value of the third associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12636,19 +11801,14 @@
           <t>mktg_promotion_intrnl_id4</t>
         </is>
       </c>
-      <c r="D383" t="inlineStr">
-        <is>
-          <t>This column contains the internal identifier for the fourth associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E383" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12668,19 +11828,14 @@
           <t>mktg_promotion_cd4</t>
         </is>
       </c>
-      <c r="D384" t="inlineStr">
-        <is>
-          <t>This column contains the code for the fourth associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12700,19 +11855,14 @@
           <t>mktg_promotion_txt4</t>
         </is>
       </c>
-      <c r="D385" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the fourth associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E385" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12732,19 +11882,14 @@
           <t>mktg_promotion_amt4</t>
         </is>
       </c>
-      <c r="D386" t="inlineStr">
-        <is>
-          <t>This column contains the monetary value of the fourth associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E386" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12764,19 +11909,14 @@
           <t>mktg_promotion_intrnl_id5</t>
         </is>
       </c>
-      <c r="D387" t="inlineStr">
-        <is>
-          <t>This column contains the internal identifier for the fifth associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12796,19 +11936,14 @@
           <t>mktg_promotion_cd5</t>
         </is>
       </c>
-      <c r="D388" t="inlineStr">
-        <is>
-          <t>This column contains the code for the fifth associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12828,19 +11963,14 @@
           <t>mktg_promotion_txt5</t>
         </is>
       </c>
-      <c r="D389" t="inlineStr">
-        <is>
-          <t>This column contains the descriptive name of the fifth associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E389" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12860,19 +11990,14 @@
           <t>mktg_promotion_amt5</t>
         </is>
       </c>
-      <c r="D390" t="inlineStr">
-        <is>
-          <t>This column contains the monetary value of the fifth associated marketing promotion.</t>
-        </is>
-      </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12892,19 +12017,14 @@
           <t>mktg_promotion_total_amt</t>
         </is>
       </c>
-      <c r="D391" t="inlineStr">
-        <is>
-          <t>This column contains the total monetary value of all applied marketing promotions.</t>
-        </is>
-      </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12924,19 +12044,14 @@
           <t>rcms_db_balance_amt</t>
         </is>
       </c>
-      <c r="D392" t="inlineStr">
-        <is>
-          <t>This column contains the remaining device balance amount from the Retail Channel Management System.</t>
-        </is>
-      </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12956,19 +12071,14 @@
           <t>rcms_bib_balance_amt</t>
         </is>
       </c>
-      <c r="D393" t="inlineStr">
-        <is>
-          <t>This column contains the remaining Bring-It-Back balance amount from the Retail Channel Management System.</t>
-        </is>
-      </c>
       <c r="E393" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -12988,19 +12098,14 @@
           <t>rcms_fin_balance_amt</t>
         </is>
       </c>
-      <c r="D394" t="inlineStr">
-        <is>
-          <t>This column contains the remaining financing balance amount from the Retail Channel Management System.</t>
-        </is>
-      </c>
       <c r="E394" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13020,19 +12125,14 @@
           <t>multi_unit_discount_amt</t>
         </is>
       </c>
-      <c r="D395" t="inlineStr">
-        <is>
-          <t>This column contains the discount amount applied for having multiple services or units on the account.</t>
-        </is>
-      </c>
       <c r="E395" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13052,19 +12152,14 @@
           <t>adjustment_reason_cd</t>
         </is>
       </c>
-      <c r="D396" t="inlineStr">
-        <is>
-          <t>This column contains a code indicating the reason for a monetary or service adjustment.</t>
-        </is>
-      </c>
       <c r="E396" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13084,19 +12179,14 @@
           <t>counter</t>
         </is>
       </c>
-      <c r="D397" t="inlineStr">
-        <is>
-          <t>This column contains a sequential number used for counting records within a transaction.</t>
-        </is>
-      </c>
       <c r="E397" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13116,19 +12206,14 @@
           <t>master_src_id</t>
         </is>
       </c>
-      <c r="D398" t="inlineStr">
-        <is>
-          <t>This column contains the identifier of the master source system from which the data originated.</t>
-        </is>
-      </c>
       <c r="E398" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13148,19 +12233,14 @@
           <t>old_device_tier_str</t>
         </is>
       </c>
-      <c r="D399" t="inlineStr">
-        <is>
-          <t>This column contains the tier classification of the customer's previous device.</t>
-        </is>
-      </c>
       <c r="E399" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13180,19 +12260,14 @@
           <t>old_device_tier_nm</t>
         </is>
       </c>
-      <c r="D400" t="inlineStr">
-        <is>
-          <t>This column contains the name of the tier classification for the customer's previous device.</t>
-        </is>
-      </c>
       <c r="E400" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13212,19 +12287,14 @@
           <t>new_device_tier_str</t>
         </is>
       </c>
-      <c r="D401" t="inlineStr">
-        <is>
-          <t>This column contains the tier classification of the customer's new device.</t>
-        </is>
-      </c>
       <c r="E401" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13244,19 +12314,14 @@
           <t>new_device_tier_nm</t>
         </is>
       </c>
-      <c r="D402" t="inlineStr">
-        <is>
-          <t>This column contains the name of the tier classification for the customer's new device.</t>
-        </is>
-      </c>
       <c r="E402" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F402" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13276,19 +12341,14 @@
           <t>old_service_tier_str</t>
         </is>
       </c>
-      <c r="D403" t="inlineStr">
-        <is>
-          <t>This column contains the tier classification of the customer's previous service plan.</t>
-        </is>
-      </c>
       <c r="E403" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13308,19 +12368,14 @@
           <t>old_service_tier_nm</t>
         </is>
       </c>
-      <c r="D404" t="inlineStr">
-        <is>
-          <t>This column contains the name of the tier classification for the customer's previous service plan.</t>
-        </is>
-      </c>
       <c r="E404" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13340,19 +12395,14 @@
           <t>new_service_tier_str</t>
         </is>
       </c>
-      <c r="D405" t="inlineStr">
-        <is>
-          <t>This column contains the tier classification of the customer's new service plan.</t>
-        </is>
-      </c>
       <c r="E405" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13372,19 +12422,14 @@
           <t>new_service_tier_nm</t>
         </is>
       </c>
-      <c r="D406" t="inlineStr">
-        <is>
-          <t>This column contains the name of the tier classification for the customer's new service plan.</t>
-        </is>
-      </c>
       <c r="E406" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13404,19 +12449,14 @@
           <t>old_price_tier_str</t>
         </is>
       </c>
-      <c r="D407" t="inlineStr">
-        <is>
-          <t>This column contains the price tier classification of the customer's previous plan.</t>
-        </is>
-      </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13436,19 +12476,14 @@
           <t>old_price_tier_nm</t>
         </is>
       </c>
-      <c r="D408" t="inlineStr">
-        <is>
-          <t>This column contains the name of the price tier classification for the customer's previous plan.</t>
-        </is>
-      </c>
       <c r="E408" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13468,19 +12503,14 @@
           <t>new_price_tier_str</t>
         </is>
       </c>
-      <c r="D409" t="inlineStr">
-        <is>
-          <t>This column contains the price tier classification of the customer's new plan.</t>
-        </is>
-      </c>
       <c r="E409" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13500,19 +12530,14 @@
           <t>new_price_tier_nm</t>
         </is>
       </c>
-      <c r="D410" t="inlineStr">
-        <is>
-          <t>This column contains the name of the price tier classification for the customer's new plan.</t>
-        </is>
-      </c>
       <c r="E410" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13532,19 +12557,14 @@
           <t>redemption_dt</t>
         </is>
       </c>
-      <c r="D411" t="inlineStr">
-        <is>
-          <t>This column contains the date on which an offer or promotion was redeemed by the customer.</t>
-        </is>
-      </c>
       <c r="E411" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F411" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13564,19 +12584,14 @@
           <t>servreq_order_id</t>
         </is>
       </c>
-      <c r="D412" t="inlineStr">
-        <is>
-          <t>This column contains the identifier for the order associated with the service request.</t>
-        </is>
-      </c>
       <c r="E412" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13596,19 +12611,14 @@
           <t>rsrvn_chnl_org_id</t>
         </is>
       </c>
-      <c r="D413" t="inlineStr">
-        <is>
-          <t>This column contains the unique identifier for the sales channel organization where a reservation was made.</t>
-        </is>
-      </c>
       <c r="E413" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13628,19 +12638,14 @@
           <t>rsrvn_chnl_org_cd</t>
         </is>
       </c>
-      <c r="D414" t="inlineStr">
-        <is>
-          <t>This column contains the code for the sales channel organization where a reservation was made.</t>
-        </is>
-      </c>
       <c r="E414" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F414" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13660,19 +12665,14 @@
           <t>rsrvn_chnl_org_txt</t>
         </is>
       </c>
-      <c r="D415" t="inlineStr">
-        <is>
-          <t>This column contains the name of the sales channel organization where a reservation was made.</t>
-        </is>
-      </c>
       <c r="E415" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13692,19 +12692,14 @@
           <t>rsrvn_outlet_id</t>
         </is>
       </c>
-      <c r="D416" t="inlineStr">
-        <is>
-          <t>This column contains the unique identifier for the sales outlet where a reservation was made.</t>
-        </is>
-      </c>
       <c r="E416" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13724,19 +12719,14 @@
           <t>rsrvn_outlet_cd</t>
         </is>
       </c>
-      <c r="D417" t="inlineStr">
-        <is>
-          <t>This column contains the code for the sales outlet where a reservation was made.</t>
-        </is>
-      </c>
       <c r="E417" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13756,19 +12746,14 @@
           <t>rsrvn_outlet_txt</t>
         </is>
       </c>
-      <c r="D418" t="inlineStr">
-        <is>
-          <t>This column contains the name of the sales outlet where a reservation was made.</t>
-        </is>
-      </c>
       <c r="E418" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13788,19 +12773,14 @@
           <t>rsrvn_sales_rep_id</t>
         </is>
       </c>
-      <c r="D419" t="inlineStr">
-        <is>
-          <t>This column contains the unique identifier for the sales representative who handled the reservation.</t>
-        </is>
-      </c>
       <c r="E419" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F419" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13820,19 +12800,14 @@
           <t>rsrvn_sales_rep_cd</t>
         </is>
       </c>
-      <c r="D420" t="inlineStr">
-        <is>
-          <t>This column contains the code for the sales representative who handled the reservation.</t>
-        </is>
-      </c>
       <c r="E420" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13852,19 +12827,14 @@
           <t>rsrvn_sales_rep_first_nm</t>
         </is>
       </c>
-      <c r="D421" t="inlineStr">
-        <is>
-          <t>This column contains the first name of the sales representative who handled the reservation.</t>
-        </is>
-      </c>
       <c r="E421" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F421" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13884,19 +12854,14 @@
           <t>rsrvn_sales_rep_last_nm</t>
         </is>
       </c>
-      <c r="D422" t="inlineStr">
-        <is>
-          <t>This column contains the last name of the sales representative who handled the reservation.</t>
-        </is>
-      </c>
       <c r="E422" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F422" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13916,19 +12881,14 @@
           <t>reference_no</t>
         </is>
       </c>
-      <c r="D423" t="inlineStr">
-        <is>
-          <t>This column contains a general reference number associated with the transaction.</t>
-        </is>
-      </c>
       <c r="E423" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F423" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13948,19 +12908,14 @@
           <t>rsrvn_txn_ts</t>
         </is>
       </c>
-      <c r="D424" t="inlineStr">
-        <is>
-          <t>This column contains the date and time the reservation transaction occurred.</t>
-        </is>
-      </c>
       <c r="E424" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F424" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -13980,19 +12935,14 @@
           <t>rsrvn_servreq_header_id</t>
         </is>
       </c>
-      <c r="D425" t="inlineStr">
-        <is>
-          <t>This column contains the service request identifier associated with the reservation.</t>
-        </is>
-      </c>
       <c r="E425" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -14012,19 +12962,14 @@
           <t>cust_hierarchy_key</t>
         </is>
       </c>
-      <c r="D426" t="inlineStr">
-        <is>
-          <t>This column contains a key that links the customer to a position within a customer hierarchy structure.</t>
-        </is>
-      </c>
       <c r="E426" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F426" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -14044,19 +12989,14 @@
           <t>cbuc_id</t>
         </is>
       </c>
-      <c r="D427" t="inlineStr">
-        <is>
-          <t>This column contains the unique identifier for the customer from the Customer Business Unit Consolidation system.</t>
-        </is>
-      </c>
       <c r="E427" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F427" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -14076,19 +13016,14 @@
           <t>rcid</t>
         </is>
       </c>
-      <c r="D428" t="inlineStr">
-        <is>
-          <t>This column contains the Regional Customer Identifier, a unique identifier for a customer within a specific region.</t>
-        </is>
-      </c>
       <c r="E428" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F428" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -14108,19 +13043,14 @@
           <t>regional_cust_nm</t>
         </is>
       </c>
-      <c r="D429" t="inlineStr">
-        <is>
-          <t>This column contains the name of the regional customer account.</t>
-        </is>
-      </c>
       <c r="E429" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F429" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -14140,19 +13070,14 @@
           <t>cbu_cust_nm</t>
         </is>
       </c>
-      <c r="D430" t="inlineStr">
-        <is>
-          <t>This column contains the name of the customer within the Customer Business Unit.</t>
-        </is>
-      </c>
       <c r="E430" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -14172,19 +13097,14 @@
           <t>cbu_cd</t>
         </is>
       </c>
-      <c r="D431" t="inlineStr">
-        <is>
-          <t>This column contains the code for the Customer Business Unit.</t>
-        </is>
-      </c>
       <c r="E431" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F431" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -14204,19 +13124,14 @@
           <t>cbu_nm</t>
         </is>
       </c>
-      <c r="D432" t="inlineStr">
-        <is>
-          <t>This column contains the name of the Customer Business Unit.</t>
-        </is>
-      </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F432" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -14236,19 +13151,14 @@
           <t>cbu_segment_type_cd</t>
         </is>
       </c>
-      <c r="D433" t="inlineStr">
-        <is>
-          <t>This column contains the customer segment code within the Customer Business Unit.</t>
-        </is>
-      </c>
       <c r="E433" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F433" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -14268,19 +13178,14 @@
           <t>cbu_subsegment_type_cd</t>
         </is>
       </c>
-      <c r="D434" t="inlineStr">
-        <is>
-          <t>This column contains the customer sub-segment code within the Customer Business Unit.</t>
-        </is>
-      </c>
       <c r="E434" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -14300,19 +13205,14 @@
           <t>new_accsry_prod_equip_cd</t>
         </is>
       </c>
-      <c r="D435" t="inlineStr">
-        <is>
-          <t>This column contains the product equipment code for a new accessory.</t>
-        </is>
-      </c>
       <c r="E435" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -14332,19 +13232,14 @@
           <t>old_accsry_prod_equip_cd</t>
         </is>
       </c>
-      <c r="D436" t="inlineStr">
-        <is>
-          <t>This column contains the product equipment code for a previous accessory.</t>
-        </is>
-      </c>
       <c r="E436" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F436" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -14364,19 +13259,14 @@
           <t>dlr_ship_to_home_ind</t>
         </is>
       </c>
-      <c r="D437" t="inlineStr">
-        <is>
-          <t>This column contains a yes/no indicator identifying if the device was shipped to the customer's home by the dealer.</t>
-        </is>
-      </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F437" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -14396,19 +13286,14 @@
           <t>sales_presence_type_cd</t>
         </is>
       </c>
-      <c r="D438" t="inlineStr">
-        <is>
-          <t>This column contains a code indicating the nature of the sales interaction, such as in-person or online.</t>
-        </is>
-      </c>
       <c r="E438" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F438" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -14428,19 +13313,14 @@
           <t>create_ts</t>
         </is>
       </c>
-      <c r="D439" t="inlineStr">
-        <is>
-          <t>This column contains the date and time the record was created in the source system.</t>
-        </is>
-      </c>
       <c r="E439" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F439" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -14460,19 +13340,14 @@
           <t>create_user_id</t>
         </is>
       </c>
-      <c r="D440" t="inlineStr">
-        <is>
-          <t>This column contains the identifier of the user or process that created the record.</t>
-        </is>
-      </c>
       <c r="E440" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F440" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -14492,19 +13367,14 @@
           <t>last_updt_ts</t>
         </is>
       </c>
-      <c r="D441" t="inlineStr">
-        <is>
-          <t>This column contains the date and time the record was last updated.</t>
-        </is>
-      </c>
       <c r="E441" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F441" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>
@@ -14524,19 +13394,14 @@
           <t>last_updt_user_id</t>
         </is>
       </c>
-      <c r="D442" t="inlineStr">
-        <is>
-          <t>This column contains the identifier of the user or process that last updated the record.</t>
-        </is>
-      </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t>gemini-2.5-pro-ca</t>
+          <t>gemma-4-saif</t>
         </is>
       </c>
       <c r="F442" t="inlineStr">
         <is>
-          <t>2026-08-18T17:09:06+00:00</t>
+          <t>2026-08-20T00:55:49+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixing collibra glossary retrieval
</commit_message>
<xml_diff>
--- a/dataplex-dq-agent/descriptions/dh1_dq_descriptions_ent_actvn.xlsx
+++ b/dataplex-dq-agent/descriptions/dh1_dq_descriptions_ent_actvn.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F462"/>
+  <dimension ref="A1:F504"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13418,17 +13418,17 @@
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>This table contains the transactional details of service requests within TELUS, capturing the various events and actions related to customer service interactions.</t>
+          <t>This table contains transactions for customer service requests, which are formal actions to activate, renew, upgrade, or cancel a customer's services.</t>
         </is>
       </c>
       <c r="E443" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13450,17 +13450,17 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>This column contains a code representing the business intelligence channel group associated with the service request.</t>
+          <t>This column contains a code used for Business Intelligence reporting to categorize the service request transaction.</t>
         </is>
       </c>
       <c r="E444" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F444" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13482,17 +13482,17 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>This column contains the billing account number associated with the service request.</t>
+          <t>This column contains the unique number assigned to the customer's billing account associated with the service request.</t>
         </is>
       </c>
       <c r="E445" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F445" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13514,17 +13514,17 @@
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>This column contains a unique identifier for the channel organization involved in the service request.</t>
+          <t>This column contains the unique identifier for the sales channel or organizational unit responsible for the service request.</t>
         </is>
       </c>
       <c r="E446" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F446" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13546,17 +13546,17 @@
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>This column contains the date and time when the record was created.</t>
+          <t>This column contains the date and time the record was created in the table.</t>
         </is>
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F447" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13578,17 +13578,17 @@
       </c>
       <c r="D448" t="inlineStr">
         <is>
-          <t>This column contains the identifier for the user who created the record.</t>
+          <t>This column contains the identifier of the user or system process that created the record.</t>
         </is>
       </c>
       <c r="E448" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F448" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13610,17 +13610,17 @@
       </c>
       <c r="D449" t="inlineStr">
         <is>
-          <t>This column contains a unique code for the dealer associated with the service request.</t>
+          <t>This column contains the code that identifies the dealer associated with the service request.</t>
         </is>
       </c>
       <c r="E449" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13642,17 +13642,17 @@
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>This column contains a unique pin for the sales representative associated with the service request.</t>
+          <t>This column contains the Personal Identification Number associated with the sales representative.</t>
         </is>
       </c>
       <c r="E450" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F450" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13674,17 +13674,17 @@
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>This column contains the date and time when the record was last updated.</t>
+          <t>This column contains the date and time the record was last updated.</t>
         </is>
       </c>
       <c r="E451" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F451" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13706,17 +13706,17 @@
       </c>
       <c r="D452" t="inlineStr">
         <is>
-          <t>This column contains the identifier for the user who last updated the record.</t>
+          <t>This column contains the identifier of the user or system process that last updated the record.</t>
         </is>
       </c>
       <c r="E452" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F452" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13738,17 +13738,17 @@
       </c>
       <c r="D453" t="inlineStr">
         <is>
-          <t>This column contains a unique identifier for the operator involved in the service request.</t>
+          <t>This column contains the unique identifier for the operator or agent who processed the service request.</t>
         </is>
       </c>
       <c r="E453" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F453" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13770,17 +13770,17 @@
       </c>
       <c r="D454" t="inlineStr">
         <is>
-          <t>This column contains a unique identifier for the outlet involved in the service request.</t>
+          <t>This column contains the unique identifier for the retail outlet or location where the service request was initiated.</t>
         </is>
       </c>
       <c r="E454" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F454" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13802,17 +13802,17 @@
       </c>
       <c r="D455" t="inlineStr">
         <is>
-          <t>This column contains a code representing the source of the registration for the service request.</t>
+          <t>This column contains a code that identifies the source system where the transaction was registered.</t>
         </is>
       </c>
       <c r="E455" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F455" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13834,17 +13834,17 @@
       </c>
       <c r="D456" t="inlineStr">
         <is>
-          <t>This column contains a unique identifier for the sales representative associated with the service request.</t>
+          <t>This column contains the unique identifier for the sales representative associated with the service request transaction.</t>
         </is>
       </c>
       <c r="E456" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F456" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13866,17 +13866,17 @@
       </c>
       <c r="D457" t="inlineStr">
         <is>
-          <t>This column contains a unique identifier for the type of event related to the service request.</t>
+          <t>This column contains a unique numeric identifier for the type of service request event, such as an activation or cancellation.</t>
         </is>
       </c>
       <c r="E457" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F457" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13898,17 +13898,17 @@
       </c>
       <c r="D458" t="inlineStr">
         <is>
-          <t>This column contains a unique identifier for the service request header.</t>
+          <t>This column contains the unique identifier for the service request.</t>
         </is>
       </c>
       <c r="E458" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F458" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13930,17 +13930,17 @@
       </c>
       <c r="D459" t="inlineStr">
         <is>
-          <t>This column contains the name of the service request header.</t>
+          <t>This column contains the name describing the type of service request.</t>
         </is>
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F459" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13962,17 +13962,17 @@
       </c>
       <c r="D460" t="inlineStr">
         <is>
-          <t>This column contains the phone number associated with the service request.</t>
+          <t>This column contains the telephone number that is the subject of the service request.</t>
         </is>
       </c>
       <c r="E460" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F460" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -13994,17 +13994,17 @@
       </c>
       <c r="D461" t="inlineStr">
         <is>
-          <t>This column contains the date and time when the service request transaction occurred.</t>
+          <t>This column contains the date and time when the service request transaction was recorded.</t>
         </is>
       </c>
       <c r="E461" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F461" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -14026,17 +14026,1351 @@
       </c>
       <c r="D462" t="inlineStr">
         <is>
-          <t>This column contains the date and time when the source service request transaction occurred.</t>
+          <t>This column contains the original date and time of the service request transaction from the source system.</t>
         </is>
       </c>
       <c r="E462" t="inlineStr">
         <is>
-          <t>mistral-small-3.2-24b</t>
+          <t>gemini-2.5-pro-ca</t>
         </is>
       </c>
       <c r="F462" t="inlineStr">
         <is>
-          <t>2026-08-20T21:16:39+00:00</t>
+          <t>2026-08-24T06:30:43+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>This table contains Master Data Management customer information, including unique customer identifiers, names, contact details such as street, municipality, province or state, country, and postal code, along with activation, deactivation, and suspension dates, and the current status of the customer, which can be active, cancelled, or suspended, and the associated line of business, such as Mobile, Fixed, or Mobile and Home, for TELUS customers.</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>mdm_cust_key</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>This column contains a unique numerical identifier for a customer within the Master Data Management system.</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>mdm_cust_id</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>This column contains a unique identifier assigned to a customer within the Master Data Management system, used to group related subscriptions for a single customer.</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>mdm_prty_id</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>This column contains a unique identifier for a party, which represents a customer, within the Master Data Management system.</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>first_nm</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>This column contains the first name of the customer.</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>last_nm</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>This column contains the last name of the customer.</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>suspend_ts</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>This column contains the timestamp when a customer's services were suspended.</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>deactivation_ts</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>This column contains the date when a customer's services were deactivated.</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>activation_ts</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>This column contains the date when a customer's services were activated.</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>initial_activation_ts</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>This column contains the date of the first activation of a customer's services.</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>mdm_status_cd</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>This column contains a code representing the current status of a customer within the Master Data Management system, such as Active, Cancelled, or Suspended.</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>line_of_business_cd</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>This column contains a code indicating the primary line of business associated with the customer, such as Mobile, Fixed, or Mobile and Home.</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>rcid_cd</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>This column contains the Regional Customer Identification code associated with the customer.</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>cbuid_cd</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>This column contains the Customer Billing Unit Identification code associated with the customer.</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>country_cd</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>This column contains a code representing the country of the customer's address.</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>civic_prov_state_cd</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>This column contains a code representing the province or state of the customer's civic address.</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>postal_cd</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>This column contains the postal code of the customer's address.</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>municipality_nm</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>This column contains the name of the municipality for the customer's address.</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>street_nm</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>This column contains the street name for the customer's address.</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>effective_start_ts</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>This column contains the timestamp when the record became effective or valid.</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>effective_end_ts</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>This column contains the timestamp when the record ceased to be effective or valid.</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>current_ind</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>This column contains an indicator that specifies if the record represents the current and most up-to-date information for the customer.</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>master_src_id</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>This column contains a unique identifier for the master source system from which the customer data originates.</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>create_ts</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>This column contains the timestamp when the record was created.</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>create_user_id</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>This column contains the identifier of the user who created the record.</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>last_updt_ts</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>This column contains the timestamp when the record was last updated.</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>bq_mdm_customer_dim</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>last_updt_user_id</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>This column contains the identifier of the user who last updated the record.</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash-ca</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>2026-08-21T22:59:40+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>bq_job_title_dim</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>This table contains the official job titles and their corresponding job functions at TELUS. A job title is the formal designation of a role.</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro-ca</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>2026-08-24T04:25:36+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>bq_job_title_dim</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>job_title_key</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>This column contains the unique system-generated identifier for each job title record.</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro-ca</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>2026-08-24T04:25:36+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>bq_job_title_dim</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>job_title_id</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>This column contains the unique identifier for a formal designation of a role.</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro-ca</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>2026-08-24T04:25:36+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>bq_job_title_dim</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>job_func_type_cd</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>This column contains a code that categorizes the business area or channel associated with the job function.</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro-ca</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>2026-08-24T04:25:36+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>bq_job_title_dim</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>job_title_nm</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>This column contains the abbreviated name for the formal designation of a role.</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro-ca</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>2026-08-24T04:25:36+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>bq_job_title_dim</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>job_title_txt</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>This column contains the full descriptive name of the role in English.</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro-ca</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>2026-08-24T04:25:36+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>bq_job_title_dim</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>job_title_fr_txt</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>This column contains the abbreviated name for the formal designation of a role in French.</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro-ca</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>2026-08-24T04:25:36+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>bq_job_title_dim</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>job_function_txt</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>This column contains the descriptive text for the associated job function in English.</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro-ca</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>2026-08-24T04:25:36+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>bq_job_title_dim</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>job_function_fr_txt</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>This column contains the descriptive text for the associated job function in French.</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro-ca</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>2026-08-24T04:25:36+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>bq_job_title_dim</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>compensation_paid_ind</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>This column contains a yes or no indicator of whether compensation is paid for the role.</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro-ca</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>2026-08-24T04:25:36+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>bq_job_title_dim</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>master_src_id</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>This column contains the unique identifier for the master source system from which the record originated.</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro-ca</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>2026-08-24T04:25:36+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>bq_job_title_dim</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>create_ts</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>This column contains the date and time when the record was created.</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro-ca</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>2026-08-24T04:25:36+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>bq_job_title_dim</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>create_user_id</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>This column contains the identifier of the user or process that created the record.</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro-ca</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>2026-08-24T04:25:36+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>bq_job_title_dim</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>last_updt_ts</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>This column contains the date and time when the record was last modified.</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro-ca</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>2026-08-24T04:25:36+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>ent_actvn</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>bq_job_title_dim</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>last_updt_user_id</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>This column contains the identifier of the user or process that last modified the record.</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>gemini-2.5-pro-ca</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>2026-08-24T04:25:36+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>